<commit_message>
style: apply ultra-sleek black color theme with glassmorphic styling
</commit_message>
<xml_diff>
--- a/automation/reports/Automation_Test_Report.xlsx
+++ b/automation/reports/Automation_Test_Report.xlsx
@@ -595,7 +595,7 @@
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>56.93s</t>
+          <t>36.49s</t>
         </is>
       </c>
     </row>
@@ -1036,7 +1036,7 @@
         </is>
       </c>
       <c r="J2" t="n">
-        <v>1.347</v>
+        <v>0.535</v>
       </c>
     </row>
     <row r="3">
@@ -1086,7 +1086,7 @@
         </is>
       </c>
       <c r="J3" t="n">
-        <v>30.898</v>
+        <v>30.189</v>
       </c>
     </row>
     <row r="4">
@@ -1136,7 +1136,7 @@
         </is>
       </c>
       <c r="J4" t="n">
-        <v>0.485</v>
+        <v>0.166</v>
       </c>
     </row>
     <row r="5">
@@ -1186,7 +1186,7 @@
         </is>
       </c>
       <c r="J5" t="n">
-        <v>0.576</v>
+        <v>0.202</v>
       </c>
     </row>
     <row r="6">
@@ -1236,7 +1236,7 @@
         </is>
       </c>
       <c r="J6" t="n">
-        <v>1.372</v>
+        <v>0.174</v>
       </c>
     </row>
     <row r="7">
@@ -1286,7 +1286,7 @@
         </is>
       </c>
       <c r="J7" t="n">
-        <v>1.274</v>
+        <v>0.14</v>
       </c>
     </row>
     <row r="8">
@@ -1336,7 +1336,7 @@
         </is>
       </c>
       <c r="J8" t="n">
-        <v>1.306</v>
+        <v>0.269</v>
       </c>
     </row>
     <row r="9">
@@ -1386,7 +1386,7 @@
         </is>
       </c>
       <c r="J9" t="n">
-        <v>0.792</v>
+        <v>0.379</v>
       </c>
     </row>
     <row r="10">
@@ -1436,7 +1436,7 @@
         </is>
       </c>
       <c r="J10" t="n">
-        <v>0.454</v>
+        <v>0.315</v>
       </c>
     </row>
     <row r="11">
@@ -1486,7 +1486,7 @@
         </is>
       </c>
       <c r="J11" t="n">
-        <v>0.912</v>
+        <v>0.291</v>
       </c>
     </row>
     <row r="12">
@@ -1536,7 +1536,7 @@
         </is>
       </c>
       <c r="J12" t="n">
-        <v>0.605</v>
+        <v>0.368</v>
       </c>
     </row>
     <row r="13">
@@ -1586,7 +1586,7 @@
         </is>
       </c>
       <c r="J13" t="n">
-        <v>0.983</v>
+        <v>0.343</v>
       </c>
     </row>
     <row r="14">
@@ -1636,7 +1636,7 @@
         </is>
       </c>
       <c r="J14" t="n">
-        <v>1.571</v>
+        <v>0.362</v>
       </c>
     </row>
     <row r="15">
@@ -1686,7 +1686,7 @@
         </is>
       </c>
       <c r="J15" t="n">
-        <v>1.932</v>
+        <v>0.496</v>
       </c>
     </row>
     <row r="16">
@@ -1736,7 +1736,7 @@
         </is>
       </c>
       <c r="J16" t="n">
-        <v>3.36</v>
+        <v>0.298</v>
       </c>
     </row>
     <row r="17">
@@ -1786,7 +1786,7 @@
         </is>
       </c>
       <c r="J17" t="n">
-        <v>1.499</v>
+        <v>0.295</v>
       </c>
     </row>
     <row r="18">
@@ -1836,7 +1836,7 @@
         </is>
       </c>
       <c r="J18" t="n">
-        <v>0.5590000000000001</v>
+        <v>0.272</v>
       </c>
     </row>
     <row r="19">
@@ -1886,7 +1886,7 @@
         </is>
       </c>
       <c r="J19" t="n">
-        <v>0.91</v>
+        <v>0.344</v>
       </c>
     </row>
     <row r="20">
@@ -1936,7 +1936,7 @@
         </is>
       </c>
       <c r="J20" t="n">
-        <v>0.704</v>
+        <v>0.111</v>
       </c>
     </row>
     <row r="21">
@@ -1986,7 +1986,7 @@
         </is>
       </c>
       <c r="J21" t="n">
-        <v>0.954</v>
+        <v>0.24</v>
       </c>
     </row>
     <row r="22">
@@ -2036,7 +2036,7 @@
         </is>
       </c>
       <c r="J22" t="n">
-        <v>1.095</v>
+        <v>0.173</v>
       </c>
     </row>
     <row r="23">
@@ -2086,7 +2086,7 @@
         </is>
       </c>
       <c r="J23" t="n">
-        <v>1.783</v>
+        <v>0.116</v>
       </c>
     </row>
     <row r="24">
@@ -2136,7 +2136,7 @@
         </is>
       </c>
       <c r="J24" t="n">
-        <v>0.837</v>
+        <v>0.145</v>
       </c>
     </row>
     <row r="25">
@@ -2186,7 +2186,7 @@
         </is>
       </c>
       <c r="J25" t="n">
-        <v>0.312</v>
+        <v>0.143</v>
       </c>
     </row>
     <row r="26">
@@ -2236,7 +2236,7 @@
         </is>
       </c>
       <c r="J26" t="n">
-        <v>0.407</v>
+        <v>0.121</v>
       </c>
     </row>
     <row r="27">
@@ -22114,7 +22114,7 @@
         </is>
       </c>
       <c r="J2" t="n">
-        <v>1.347</v>
+        <v>0.535</v>
       </c>
     </row>
     <row r="3">
@@ -22164,7 +22164,7 @@
         </is>
       </c>
       <c r="J3" t="n">
-        <v>30.898</v>
+        <v>30.189</v>
       </c>
     </row>
     <row r="4">
@@ -22214,7 +22214,7 @@
         </is>
       </c>
       <c r="J4" t="n">
-        <v>0.485</v>
+        <v>0.166</v>
       </c>
     </row>
     <row r="5">
@@ -22264,7 +22264,7 @@
         </is>
       </c>
       <c r="J5" t="n">
-        <v>0.576</v>
+        <v>0.202</v>
       </c>
     </row>
     <row r="6">
@@ -22314,7 +22314,7 @@
         </is>
       </c>
       <c r="J6" t="n">
-        <v>1.372</v>
+        <v>0.174</v>
       </c>
     </row>
     <row r="7">
@@ -22364,7 +22364,7 @@
         </is>
       </c>
       <c r="J7" t="n">
-        <v>1.274</v>
+        <v>0.14</v>
       </c>
     </row>
     <row r="8">
@@ -22414,7 +22414,7 @@
         </is>
       </c>
       <c r="J8" t="n">
-        <v>1.306</v>
+        <v>0.269</v>
       </c>
     </row>
     <row r="9">
@@ -22464,7 +22464,7 @@
         </is>
       </c>
       <c r="J9" t="n">
-        <v>0.792</v>
+        <v>0.379</v>
       </c>
     </row>
     <row r="10">
@@ -22514,7 +22514,7 @@
         </is>
       </c>
       <c r="J10" t="n">
-        <v>0.454</v>
+        <v>0.315</v>
       </c>
     </row>
     <row r="11">
@@ -22564,7 +22564,7 @@
         </is>
       </c>
       <c r="J11" t="n">
-        <v>0.912</v>
+        <v>0.291</v>
       </c>
     </row>
     <row r="12">
@@ -22614,7 +22614,7 @@
         </is>
       </c>
       <c r="J12" t="n">
-        <v>0.605</v>
+        <v>0.368</v>
       </c>
     </row>
     <row r="13">
@@ -22664,7 +22664,7 @@
         </is>
       </c>
       <c r="J13" t="n">
-        <v>0.983</v>
+        <v>0.343</v>
       </c>
     </row>
     <row r="14">
@@ -22714,7 +22714,7 @@
         </is>
       </c>
       <c r="J14" t="n">
-        <v>1.571</v>
+        <v>0.362</v>
       </c>
     </row>
     <row r="15">
@@ -22764,7 +22764,7 @@
         </is>
       </c>
       <c r="J15" t="n">
-        <v>1.932</v>
+        <v>0.496</v>
       </c>
     </row>
     <row r="16">
@@ -22814,7 +22814,7 @@
         </is>
       </c>
       <c r="J16" t="n">
-        <v>3.36</v>
+        <v>0.298</v>
       </c>
     </row>
     <row r="17">
@@ -22864,7 +22864,7 @@
         </is>
       </c>
       <c r="J17" t="n">
-        <v>1.499</v>
+        <v>0.295</v>
       </c>
     </row>
     <row r="18">
@@ -22914,7 +22914,7 @@
         </is>
       </c>
       <c r="J18" t="n">
-        <v>0.5590000000000001</v>
+        <v>0.272</v>
       </c>
     </row>
     <row r="19">
@@ -22964,7 +22964,7 @@
         </is>
       </c>
       <c r="J19" t="n">
-        <v>0.91</v>
+        <v>0.344</v>
       </c>
     </row>
     <row r="20">
@@ -23014,7 +23014,7 @@
         </is>
       </c>
       <c r="J20" t="n">
-        <v>0.704</v>
+        <v>0.111</v>
       </c>
     </row>
     <row r="21">
@@ -23064,7 +23064,7 @@
         </is>
       </c>
       <c r="J21" t="n">
-        <v>0.954</v>
+        <v>0.24</v>
       </c>
     </row>
     <row r="22">
@@ -23114,7 +23114,7 @@
         </is>
       </c>
       <c r="J22" t="n">
-        <v>1.095</v>
+        <v>0.173</v>
       </c>
     </row>
     <row r="23">
@@ -23164,7 +23164,7 @@
         </is>
       </c>
       <c r="J23" t="n">
-        <v>1.783</v>
+        <v>0.116</v>
       </c>
     </row>
     <row r="24">
@@ -23214,7 +23214,7 @@
         </is>
       </c>
       <c r="J24" t="n">
-        <v>0.837</v>
+        <v>0.145</v>
       </c>
     </row>
     <row r="25">
@@ -23264,7 +23264,7 @@
         </is>
       </c>
       <c r="J25" t="n">
-        <v>0.312</v>
+        <v>0.143</v>
       </c>
     </row>
     <row r="26">
@@ -23314,7 +23314,7 @@
         </is>
       </c>
       <c r="J26" t="n">
-        <v>0.407</v>
+        <v>0.121</v>
       </c>
     </row>
     <row r="27">

</xml_diff>